<commit_message>
Correction finalement assez mineure pour distinguer les importations et les...
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
+++ b/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
@@ -438,9 +438,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -462,9 +460,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -493,9 +489,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -503,9 +497,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -513,9 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -548,31 +538,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Business as usual</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
@@ -589,8 +579,6 @@
           <t>M inhabitant</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>INSEE data</t>
@@ -608,8 +596,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Logistic</t>
@@ -627,8 +613,6 @@
           <t>kgN/cap/yr</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -646,8 +630,6 @@
           <t>kgN/cap/yr</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -665,8 +647,6 @@
           <t>kgN/cap/yr</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -684,8 +664,6 @@
           <t>ha</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -703,8 +681,6 @@
           <t>ha</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -714,7 +690,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Net import of vegetal pdcts</t>
+          <t>Import of vegetal pdcts</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -722,66 +698,75 @@
           <t>ktN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Historical trend. Used as a goal but may be adjusted according to territory situation</t>
+          <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Total LU</t>
+          <t>Export of vegetal pdcts</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LU</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>ktN</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Historical trend, see prop for each livestock in technical sheet</t>
+          <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Synth N fertilizer application to cropland</t>
+          <t>Total LU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>kgN/ha/yr</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+          <t>LU</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>No business as usual: computed with optimization model to fertilize all crops</t>
+          <t>Historical trend, see prop for each livestock in technical sheet</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Synth N fertilizer application to cropland</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>kgN/ha/yr</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No business as usual: computed with optimization model to fertilize all crops</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Synth N fertilizer application to grassland</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>kgN/ha/yr</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>No business as usual: computed with optimization model to fertilize all crops</t>
         </is>
@@ -1609,7 +1594,6 @@
           <t xml:space="preserve">Natural meadow </t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="b">
         <v>0</v>
       </c>
@@ -1634,31 +1618,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Business as usual</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
@@ -1670,11 +1654,9 @@
           <t>Weight diet</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Weight for the optimization model</t>
@@ -1687,11 +1669,9 @@
           <t>Weight synthetic fertilizer use</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>5</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Weight for the optimization model</t>
@@ -1701,14 +1681,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Weight import/export balance</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>Weight import</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>2</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Weight for the optimization model</t>
@@ -1718,26 +1696,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in urban area</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+          <t>Weight export</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Weight for the optimization model</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in rural area</t>
+          <t>N recycling rate of human excretion in urban area</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1745,8 +1719,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1756,7 +1728,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
+          <t>N recycling rate of human excretion in rural area</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1764,8 +1736,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1775,7 +1745,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1783,8 +1753,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1794,26 +1762,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>kgN excreted by bovines LU</t>
+          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>kgN</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>%</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Historical trend</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>kgN excreted by equines LU</t>
+          <t>kgN excreted by bovines LU</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1821,8 +1787,6 @@
           <t>kgN</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -1832,7 +1796,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>kgN excreted by caprines LU</t>
+          <t>kgN excreted by equines LU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1840,8 +1804,6 @@
           <t>kgN</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -1851,7 +1813,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>kgN excreted by ovines LU</t>
+          <t>kgN excreted by caprines LU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1859,8 +1821,6 @@
           <t>kgN</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -1870,7 +1830,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>kgN excreted by porcines LU</t>
+          <t>kgN excreted by ovines LU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1878,8 +1838,6 @@
           <t>kgN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -1889,7 +1847,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kgN excreted by poultry LU</t>
+          <t>kgN excreted by porcines LU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1897,8 +1855,6 @@
           <t>kgN</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Historical trend</t>
@@ -1908,26 +1864,24 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bovines % excretion on grassland</t>
+          <t>kgN excreted by poultry LU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+          <t>kgN</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Historical trend</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as litter manure</t>
+          <t>Bovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1935,8 +1889,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1946,7 +1898,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as other manure</t>
+          <t>Bovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1954,8 +1906,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1965,7 +1915,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as slurry</t>
+          <t>Bovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1973,8 +1923,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -1984,7 +1932,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ovines % excretion on grassland</t>
+          <t>Bovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1992,8 +1940,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2003,7 +1949,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as litter manure</t>
+          <t>Ovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2011,8 +1957,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2022,7 +1966,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as other manure</t>
+          <t>Ovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2030,8 +1974,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2041,7 +1983,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as slurry</t>
+          <t>Ovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2049,8 +1991,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2060,7 +2000,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Equines % excretion on grassland</t>
+          <t>Ovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2068,8 +2008,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2079,7 +2017,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as litter manure</t>
+          <t>Equines % excretion on grassland</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2087,8 +2025,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2098,7 +2034,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as other manure</t>
+          <t>Equines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2106,8 +2042,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2117,7 +2051,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as slurry</t>
+          <t>Equines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2125,8 +2059,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2136,7 +2068,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Caprines % excretion on grassland</t>
+          <t>Equines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2144,8 +2076,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2155,7 +2085,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as litter manure</t>
+          <t>Caprines % excretion on grassland</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2163,8 +2093,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2174,7 +2102,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as other manure</t>
+          <t>Caprines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2182,8 +2110,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2193,7 +2119,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as slurry</t>
+          <t>Caprines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2201,8 +2127,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2212,7 +2136,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Porcines % excretion on grassland</t>
+          <t>Caprines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2220,8 +2144,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2231,7 +2153,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as litter manure</t>
+          <t>Porcines % excretion on grassland</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2239,8 +2161,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2250,7 +2170,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as other manure</t>
+          <t>Porcines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2258,8 +2178,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2269,7 +2187,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as slurry</t>
+          <t>Porcines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2277,8 +2195,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2288,7 +2204,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Poultry % excretion on grassland</t>
+          <t>Porcines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2296,8 +2212,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2307,7 +2221,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as litter manure</t>
+          <t>Poultry % excretion on grassland</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2315,8 +2229,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2326,7 +2238,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as other manure</t>
+          <t>Poultry % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2334,8 +2246,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2345,7 +2255,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as slurry</t>
+          <t>Poultry % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2353,8 +2263,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2364,16 +2272,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bovines LU</t>
+          <t>Poultry % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>prop</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+          <t>%</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2383,7 +2289,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ovines LU</t>
+          <t>Bovines LU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2391,8 +2297,6 @@
           <t>prop</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2402,7 +2306,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Caprines LU</t>
+          <t>Ovines LU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2410,8 +2314,6 @@
           <t>prop</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2421,7 +2323,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Equines LU</t>
+          <t>Caprines LU</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2429,8 +2331,6 @@
           <t>prop</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2440,7 +2340,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Porcines LU</t>
+          <t>Equines LU</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2448,8 +2348,6 @@
           <t>prop</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2459,7 +2357,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Poultry LU</t>
+          <t>Porcines LU</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,8 +2365,6 @@
           <t>prop</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
@@ -2478,26 +2374,24 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Bovines productivity</t>
+          <t>Poultry LU</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>kgcarcass/LU</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+          <t>prop</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ovines productivity</t>
+          <t>Bovines productivity</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2505,8 +2399,6 @@
           <t>kgcarcass/LU</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2516,7 +2408,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Caprines productivity</t>
+          <t>Ovines productivity</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2524,8 +2416,6 @@
           <t>kgcarcass/LU</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2535,7 +2425,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Equines productivity</t>
+          <t>Caprines productivity</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2543,8 +2433,6 @@
           <t>kgcarcass/LU</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2554,7 +2442,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Porcines productivity</t>
+          <t>Equines productivity</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2562,8 +2450,6 @@
           <t>kgcarcass/LU</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2573,7 +2459,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Poultry productivity</t>
+          <t>Porcines productivity</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2581,8 +2467,6 @@
           <t>kgcarcass/LU</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2592,16 +2476,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Bovines dairy productivity</t>
+          <t>Poultry productivity</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>kg/LU</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
+          <t>kgcarcass/LU</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2611,7 +2493,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ovines dairy productivity</t>
+          <t>Bovines dairy productivity</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2619,8 +2501,6 @@
           <t>kg/LU</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2630,7 +2510,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Caprines dairy productivity</t>
+          <t>Ovines dairy productivity</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2638,8 +2518,6 @@
           <t>kg/LU</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
@@ -2649,17 +2527,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Caprines dairy productivity</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>kg/LU</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>Poultry dairy productivity</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>kg/LU</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>

</xml_diff>

<commit_message>
Added lines for methanizer in main and technical scenario sheets
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
+++ b/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
@@ -438,7 +438,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -460,7 +459,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -489,7 +487,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -497,7 +494,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -505,7 +501,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -538,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -769,6 +764,23 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>No business as usual: computed with optimization model to fertilize all crops</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Methaniser production</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>GWh/yr</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Regional 2021 data mapped on 2006 33 region plant production. Used as a goal but may be adjusted according to territory situation</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1655,7 +1667,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1711,24 +1723,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in urban area</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+          <t>Weight energy</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Weight for the optimization model</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in rural area</t>
+          <t>N recycling rate of human excretion in urban area</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1745,7 +1755,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
+          <t>N recycling rate of human excretion in rural area</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1762,7 +1772,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1779,24 +1789,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>kgN excreted by bovines LU</t>
+          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>kgN</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Historical trend</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>kgN excreted by equines LU</t>
+          <t>kgN excreted by bovines LU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1813,7 +1823,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>kgN excreted by caprines LU</t>
+          <t>kgN excreted by equines LU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1830,7 +1840,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>kgN excreted by ovines LU</t>
+          <t>kgN excreted by caprines LU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1847,7 +1857,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kgN excreted by porcines LU</t>
+          <t>kgN excreted by ovines LU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1864,7 +1874,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>kgN excreted by poultry LU</t>
+          <t>kgN excreted by porcines LU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1881,24 +1891,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bovines % excretion on grassland</t>
+          <t>kgN excreted by poultry LU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kgN</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Historical trend</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as litter manure</t>
+          <t>Bovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1915,7 +1925,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as other manure</t>
+          <t>Bovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1932,7 +1942,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as slurry</t>
+          <t>Bovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1949,7 +1959,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ovines % excretion on grassland</t>
+          <t>Bovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1966,7 +1976,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as litter manure</t>
+          <t>Ovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1983,7 +1993,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as other manure</t>
+          <t>Ovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2000,7 +2010,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as slurry</t>
+          <t>Ovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2017,7 +2027,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Equines % excretion on grassland</t>
+          <t>Ovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2034,7 +2044,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as litter manure</t>
+          <t>Equines % excretion on grassland</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2051,7 +2061,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as other manure</t>
+          <t>Equines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2068,7 +2078,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as slurry</t>
+          <t>Equines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2085,7 +2095,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Caprines % excretion on grassland</t>
+          <t>Equines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2102,7 +2112,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as litter manure</t>
+          <t>Caprines % excretion on grassland</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2119,7 +2129,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as other manure</t>
+          <t>Caprines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2136,7 +2146,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as slurry</t>
+          <t>Caprines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2153,7 +2163,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Porcines % excretion on grassland</t>
+          <t>Caprines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2170,7 +2180,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as litter manure</t>
+          <t>Porcines % excretion on grassland</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2187,7 +2197,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as other manure</t>
+          <t>Porcines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2204,7 +2214,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as slurry</t>
+          <t>Porcines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2221,7 +2231,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Poultry % excretion on grassland</t>
+          <t>Porcines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2238,7 +2248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as litter manure</t>
+          <t>Poultry % excretion on grassland</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2255,7 +2265,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as other manure</t>
+          <t>Poultry % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2272,7 +2282,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as slurry</t>
+          <t>Poultry % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2289,12 +2299,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bovines LU</t>
+          <t>Poultry % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2306,7 +2316,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ovines LU</t>
+          <t>Bovines LU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2323,7 +2333,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Caprines LU</t>
+          <t>Ovines LU</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2340,7 +2350,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Equines LU</t>
+          <t>Caprines LU</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2357,7 +2367,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Porcines LU</t>
+          <t>Equines LU</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2374,7 +2384,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Poultry LU</t>
+          <t>Porcines LU</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2391,24 +2401,24 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bovines productivity</t>
+          <t>Poultry LU</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>kgcarcass/LU</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ovines productivity</t>
+          <t>Bovines productivity</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2425,7 +2435,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Caprines productivity</t>
+          <t>Ovines productivity</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2442,7 +2452,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Equines productivity</t>
+          <t>Caprines productivity</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2459,7 +2469,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Porcines productivity</t>
+          <t>Equines productivity</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2476,7 +2486,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Poultry productivity</t>
+          <t>Porcines productivity</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2493,12 +2503,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bovines dairy productivity</t>
+          <t>Poultry productivity</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>kg/LU</t>
+          <t>kgcarcass/LU</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2510,7 +2520,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ovines dairy productivity</t>
+          <t>Bovines dairy productivity</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2527,7 +2537,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Caprines dairy productivity</t>
+          <t>Ovines dairy productivity</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2544,15 +2554,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>Caprines dairy productivity</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>kg/LU</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Poultry dairy productivity</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>kg/LU</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>

</xml_diff>

<commit_message>
Added prop input for methanisers and weght for methanizer in scenario
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
+++ b/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
@@ -1630,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1738,24 +1738,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in urban area</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+          <t>Weight methaniser input</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>25</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Weight for the optimization model</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in rural area</t>
+          <t>N recycling rate of human excretion in urban area</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1772,7 +1770,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
+          <t>N recycling rate of human excretion in rural area</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1789,7 +1787,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1806,24 +1804,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>kgN excreted by bovines LU</t>
+          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>kgN</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Historical trend</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>kgN excreted by equines LU</t>
+          <t>kgN excreted by bovines LU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1840,7 +1838,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>kgN excreted by caprines LU</t>
+          <t>kgN excreted by equines LU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1857,7 +1855,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kgN excreted by ovines LU</t>
+          <t>kgN excreted by caprines LU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1874,7 +1872,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>kgN excreted by porcines LU</t>
+          <t>kgN excreted by ovines LU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1891,7 +1889,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kgN excreted by poultry LU</t>
+          <t>kgN excreted by porcines LU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1908,24 +1906,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bovines % excretion on grassland</t>
+          <t>kgN excreted by poultry LU</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kgN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Historical trend</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as litter manure</t>
+          <t>Bovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1942,7 +1940,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as other manure</t>
+          <t>Bovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1959,7 +1957,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as slurry</t>
+          <t>Bovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1976,7 +1974,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ovines % excretion on grassland</t>
+          <t>Bovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1993,7 +1991,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as litter manure</t>
+          <t>Ovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2010,7 +2008,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as other manure</t>
+          <t>Ovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2027,7 +2025,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as slurry</t>
+          <t>Ovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2044,7 +2042,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Equines % excretion on grassland</t>
+          <t>Ovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2061,7 +2059,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as litter manure</t>
+          <t>Equines % excretion on grassland</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2078,7 +2076,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as other manure</t>
+          <t>Equines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2095,7 +2093,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as slurry</t>
+          <t>Equines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2112,7 +2110,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Caprines % excretion on grassland</t>
+          <t>Equines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2129,7 +2127,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as litter manure</t>
+          <t>Caprines % excretion on grassland</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2146,7 +2144,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as other manure</t>
+          <t>Caprines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2163,7 +2161,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as slurry</t>
+          <t>Caprines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2180,7 +2178,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Porcines % excretion on grassland</t>
+          <t>Caprines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2197,7 +2195,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as litter manure</t>
+          <t>Porcines % excretion on grassland</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2214,7 +2212,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as other manure</t>
+          <t>Porcines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2231,7 +2229,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as slurry</t>
+          <t>Porcines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2248,7 +2246,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Poultry % excretion on grassland</t>
+          <t>Porcines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2265,7 +2263,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as litter manure</t>
+          <t>Poultry % excretion on grassland</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2282,7 +2280,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as other manure</t>
+          <t>Poultry % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2299,7 +2297,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as slurry</t>
+          <t>Poultry % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2316,12 +2314,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bovines LU</t>
+          <t>Poultry % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2333,7 +2331,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ovines LU</t>
+          <t>Bovines LU</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2350,7 +2348,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Caprines LU</t>
+          <t>Ovines LU</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2367,7 +2365,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Equines LU</t>
+          <t>Caprines LU</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2384,7 +2382,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Porcines LU</t>
+          <t>Equines LU</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2401,7 +2399,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Poultry LU</t>
+          <t>Porcines LU</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2418,24 +2416,24 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bovines productivity</t>
+          <t>Poultry LU</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>kgcarcass/LU</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ovines productivity</t>
+          <t>Bovines productivity</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2452,7 +2450,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Caprines productivity</t>
+          <t>Ovines productivity</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2469,7 +2467,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Equines productivity</t>
+          <t>Caprines productivity</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2486,7 +2484,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Porcines productivity</t>
+          <t>Equines productivity</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2503,7 +2501,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Poultry productivity</t>
+          <t>Porcines productivity</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2520,12 +2518,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Bovines dairy productivity</t>
+          <t>Poultry productivity</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>kg/LU</t>
+          <t>kgcarcass/LU</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2537,7 +2535,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ovines dairy productivity</t>
+          <t>Bovines dairy productivity</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2554,7 +2552,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Caprines dairy productivity</t>
+          <t>Ovines dairy productivity</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2571,17 +2569,134 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Caprines dairy productivity</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>kg/LU</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>Poultry dairy productivity</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>kg/LU</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Share of crop residues in methaniser</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Share of green waste in methaniser</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Share of dedicated culture in methaniser</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Share of animal food industry in methaniser</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Share of livestock effluent in methaniser</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout des nouveaux excel.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
+++ b/src/grafs_e/data/scenario_region/Exponential/Ain-Rhône.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,24 +583,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Urban population</t>
+          <t>Total per capita protein ingestion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kgN/cap/yr</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Logistic</t>
+          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Total per capita protein ingestion</t>
+          <t>Vegetal per capita protein ingestion</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vegetal per capita protein ingestion</t>
+          <t>Edible animal per capita protein ingestion (excl fish)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -634,24 +634,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Edible animal per capita protein ingestion (excl fish)</t>
+          <t>Arable area</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>kgN/cap/yr</t>
+          <t>ha</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
+          <t>Historical trend</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arable area</t>
+          <t>Permanent grassland area</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -668,24 +668,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Permanent grassland area</t>
+          <t>Import of vegetal pdcts</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ha</t>
+          <t>ktN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Historical trend</t>
+          <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Import of vegetal pdcts</t>
+          <t>Export of vegetal pdcts</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -702,41 +702,41 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Export of vegetal pdcts</t>
+          <t>Total LU</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ktN</t>
+          <t>LU</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2006 data. Used as a goal but may be adjusted according to territory situation</t>
+          <t>Historical trend, see prop for each livestock in technical sheet</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Total LU</t>
+          <t>Synth N fertilizer application to cropland</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>kgN/ha/yr</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Historical trend, see prop for each livestock in technical sheet</t>
+          <t>No business as usual: computed with optimization model to fertilize all crops</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Synth N fertilizer application to cropland</t>
+          <t>Synth N fertilizer application to grassland</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -753,32 +753,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Synth N fertilizer application to grassland</t>
+          <t>Methaniser production</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>kgN/ha/yr</t>
+          <t>GWh/yr</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>No business as usual: computed with optimization model to fertilize all crops</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Methaniser production</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>GWh/yr</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
         <is>
           <t>Regional 2021 data mapped on 2006 33 region plant production. Used as a goal but may be adjusted according to territory situation</t>
         </is>
@@ -1630,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1659,6 +1642,11 @@
           <t>Comment</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1674,6 +1662,9 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1689,6 +1680,9 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1704,6 +1698,9 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1719,6 +1716,9 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1734,6 +1734,9 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1749,28 +1752,31 @@
           <t>Weight for the optimization model</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in urban area</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+          <t>Urban population</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Logistic</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>%</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Taken as the last historical value</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>N recycling rate of human excretion in rural area</t>
+          <t>N recycling rate of human excretion in urban area</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1782,12 +1788,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F9" t="n">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
+          <t>N recycling rate of human excretion in rural area</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1799,12 +1808,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F10" t="n">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
+          <t>NH3 volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1816,29 +1828,35 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F11" t="n">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>kgN excreted by bovines LU</t>
+          <t>Indirect N2O volatilization coefficient for synthetic nitrogen</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>kgN</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Historical trend</t>
-        </is>
+          <t>Taken as the last historical value</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>kgN excreted by equines LU</t>
+          <t>kgN excreted by bovines LU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1850,12 +1868,15 @@
         <is>
           <t>Historical trend</t>
         </is>
+      </c>
+      <c r="F13" t="n">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kgN excreted by caprines LU</t>
+          <t>kgN excreted by equines LU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1867,12 +1888,15 @@
         <is>
           <t>Historical trend</t>
         </is>
+      </c>
+      <c r="F14" t="n">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>kgN excreted by ovines LU</t>
+          <t>kgN excreted by caprines LU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1884,12 +1908,15 @@
         <is>
           <t>Historical trend</t>
         </is>
+      </c>
+      <c r="F15" t="n">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kgN excreted by porcines LU</t>
+          <t>kgN excreted by ovines LU</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1901,12 +1928,15 @@
         <is>
           <t>Historical trend</t>
         </is>
+      </c>
+      <c r="F16" t="n">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>kgN excreted by poultry LU</t>
+          <t>kgN excreted by porcines LU</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1918,29 +1948,35 @@
         <is>
           <t>Historical trend</t>
         </is>
+      </c>
+      <c r="F17" t="n">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bovines % excretion on grassland</t>
+          <t>kgN excreted by poultry LU</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kgN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Taken as the last historical value</t>
-        </is>
+          <t>Historical trend</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as litter manure</t>
+          <t>Bovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1952,12 +1988,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F19" t="n">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as other manure</t>
+          <t>Bovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1969,12 +2008,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F20" t="n">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bovines % excretion in the barn as slurry</t>
+          <t>Bovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1986,12 +2028,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F21" t="n">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ovines % excretion on grassland</t>
+          <t>Bovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2003,12 +2048,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F22" t="n">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as litter manure</t>
+          <t>Ovines % excretion on grassland</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2020,12 +2068,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F23" t="n">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as other manure</t>
+          <t>Ovines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2037,12 +2088,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F24" t="n">
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ovines % excretion in the barn as slurry</t>
+          <t>Ovines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2054,12 +2108,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F25" t="n">
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Equines % excretion on grassland</t>
+          <t>Ovines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2071,12 +2128,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F26" t="n">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as litter manure</t>
+          <t>Equines % excretion on grassland</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2088,12 +2148,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F27" t="n">
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as other manure</t>
+          <t>Equines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2105,12 +2168,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F28" t="n">
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Equines % excretion in the barn as slurry</t>
+          <t>Equines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2122,12 +2188,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F29" t="n">
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Caprines % excretion on grassland</t>
+          <t>Equines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2139,12 +2208,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F30" t="n">
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as litter manure</t>
+          <t>Caprines % excretion on grassland</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2156,12 +2228,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F31" t="n">
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as other manure</t>
+          <t>Caprines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2173,12 +2248,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F32" t="n">
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Caprines % excretion in the barn as slurry</t>
+          <t>Caprines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2190,12 +2268,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F33" t="n">
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Porcines % excretion on grassland</t>
+          <t>Caprines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2207,12 +2288,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F34" t="n">
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as litter manure</t>
+          <t>Porcines % excretion on grassland</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2224,12 +2308,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F35" t="n">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as other manure</t>
+          <t>Porcines % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2241,12 +2328,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F36" t="n">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Porcines % excretion in the barn as slurry</t>
+          <t>Porcines % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2258,12 +2348,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F37" t="n">
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Poultry % excretion on grassland</t>
+          <t>Porcines % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2275,12 +2368,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F38" t="n">
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as litter manure</t>
+          <t>Poultry % excretion on grassland</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2292,12 +2388,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F39" t="n">
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as other manure</t>
+          <t>Poultry % excretion in the barn as litter manure</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2309,12 +2408,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F40" t="n">
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Poultry % excretion in the barn as slurry</t>
+          <t>Poultry % excretion in the barn as other manure</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,29 +2428,35 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F41" t="n">
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Bovines LU</t>
+          <t>Poultry % excretion in the barn as slurry</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F42" t="n">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ovines LU</t>
+          <t>Bovines LU</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2360,12 +2468,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F43" t="n">
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Caprines LU</t>
+          <t>Ovines LU</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2377,12 +2488,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F44" t="n">
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Equines LU</t>
+          <t>Caprines LU</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2394,12 +2508,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F45" t="n">
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Porcines LU</t>
+          <t>Equines LU</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2411,12 +2528,15 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F46" t="n">
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Poultry LU</t>
+          <t>Porcines LU</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2428,29 +2548,35 @@
         <is>
           <t>Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F47" t="n">
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bovines productivity</t>
+          <t>Poultry LU</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>kgcarcass/LU</t>
+          <t>prop</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
-        </is>
+          <t>Taken as the last historical value</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ovines productivity</t>
+          <t>Bovines productivity</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2462,12 +2588,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F49" t="n">
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Caprines productivity</t>
+          <t>Ovines productivity</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2479,12 +2608,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F50" t="n">
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Equines productivity</t>
+          <t>Caprines productivity</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2496,12 +2628,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F51" t="n">
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Porcines productivity</t>
+          <t>Equines productivity</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2513,12 +2648,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F52" t="n">
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Poultry productivity</t>
+          <t>Porcines productivity</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2530,29 +2668,35 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F53" t="n">
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bovines dairy productivity</t>
+          <t>Poultry productivity</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>kg/LU</t>
+          <t>kgcarcass/LU</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F54" t="n">
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ovines dairy productivity</t>
+          <t>Bovines dairy productivity</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2564,12 +2708,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F55" t="n">
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Caprines dairy productivity</t>
+          <t>Ovines dairy productivity</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2581,12 +2728,15 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F56" t="n">
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Poultry dairy productivity</t>
+          <t>Caprines dairy productivity</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2598,32 +2748,35 @@
         <is>
           <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
         </is>
+      </c>
+      <c r="F57" t="n">
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Share of crop residues in methaniser</t>
+          <t>Poultry dairy productivity</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>prop</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>0.06</v>
+          <t>kg/LU</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Adapted from ONRB data</t>
-        </is>
+          <t>These groups are taken as a whole even if only a part is producing meat, milk or eggs. Taken as the last historical value</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Share of green waste in methaniser</t>
+          <t>Share of crop residues in methaniser</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2632,18 +2785,21 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>Adapted from ONRB data</t>
         </is>
+      </c>
+      <c r="F59" t="n">
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Share of dedicated culture in methaniser</t>
+          <t>Share of green waste in methaniser</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2652,18 +2808,21 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.09</v>
+        <v>0.02</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
           <t>Adapted from ONRB data</t>
         </is>
+      </c>
+      <c r="F60" t="n">
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Share of animal food industry in methaniser</t>
+          <t>Share of dedicated culture in methaniser</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2672,32 +2831,61 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>Adapted from ONRB data</t>
         </is>
+      </c>
+      <c r="F61" t="n">
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>Share of animal food industry in methaniser</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Adapted from ONRB data</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>Share of livestock effluent in methaniser</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>prop</t>
         </is>
       </c>
-      <c r="C62" t="n">
+      <c r="C63" t="n">
         <v>0.79</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Adapted from ONRB data</t>
         </is>
+      </c>
+      <c r="F63" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>